<commit_message>
Add Streamlit app and SQLite backend
</commit_message>
<xml_diff>
--- a/lista_palabras.xlsx
+++ b/lista_palabras.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Startklar\Documents\PythonProjects\deutsch-wortschatz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{777DE3E3-3796-45A8-A0AB-1C59E2E29C8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6579B133-80E1-423F-9959-BB125B12664D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$131</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$130</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="563">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="562">
   <si>
     <t>word</t>
   </si>
@@ -884,9 +884,6 @@
   </si>
   <si>
     <t>Er benehmt sich gut.</t>
-  </si>
-  <si>
-    <t>imprudentemente; insensatamente</t>
   </si>
   <si>
     <t>erbarmungslos</t>
@@ -1767,7 +1764,18 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -2065,7 +2073,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G131"/>
+  <dimension ref="A1:G130"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14.3984375" style="2" bestFit="1" customWidth="1"/>
@@ -2103,82 +2111,82 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>516</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>517</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>384</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>385</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>386</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>469</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>471</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>472</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>507</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>508</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>509</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>510</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
@@ -2203,47 +2211,47 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>408</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>326</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>186</v>
@@ -2252,33 +2260,33 @@
         <v>187</v>
       </c>
       <c r="E9" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>363</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>364</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>537</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>451</v>
-      </c>
-      <c r="F10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>538</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>539</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
@@ -2320,22 +2328,22 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D13" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="G13" s="2" t="s">
         <v>373</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
@@ -2431,22 +2439,22 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D19" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>350</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>351</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.45">
@@ -2471,22 +2479,22 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D21" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="F21" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="G21" s="2" t="s">
         <v>356</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
@@ -2508,7 +2516,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>186</v>
@@ -2517,13 +2525,13 @@
         <v>269</v>
       </c>
       <c r="E23" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>337</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="G23" s="2" t="s">
         <v>338</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
@@ -2545,7 +2553,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>186</v>
@@ -2554,30 +2562,30 @@
         <v>187</v>
       </c>
       <c r="E25" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>494</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="G25" s="2" t="s">
         <v>495</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E26" s="2" t="s">
+      <c r="F26" s="2" t="s">
         <v>432</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="G26" s="2" t="s">
         <v>433</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>434</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.45">
@@ -2619,22 +2627,22 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D29" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="E29" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="F29" s="2" t="s">
         <v>555</v>
       </c>
-      <c r="F29" s="2" t="s">
+      <c r="G29" s="2" t="s">
         <v>556</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>557</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.45">
@@ -2676,7 +2684,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>186</v>
@@ -2685,144 +2693,144 @@
         <v>187</v>
       </c>
       <c r="E32" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>428</v>
       </c>
-      <c r="F32" s="2" t="s">
+      <c r="G32" s="2" t="s">
         <v>429</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>379</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E33" s="2" t="s">
+      <c r="F33" s="2" t="s">
         <v>380</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="G33" s="2" t="s">
         <v>381</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>382</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D34" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>545</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="F34" s="2" t="s">
         <v>546</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="G34" s="2" t="s">
         <v>547</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>548</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>540</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E35" s="2" t="s">
+      <c r="F35" s="2" t="s">
         <v>541</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="G35" s="2" t="s">
         <v>542</v>
-      </c>
-      <c r="G35" s="2" t="s">
-        <v>543</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D36" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="E36" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="F36" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="F36" s="2" t="s">
+      <c r="G36" s="2" t="s">
         <v>334</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E37" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E37" s="2" t="s">
+      <c r="F37" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="F37" s="2" t="s">
+      <c r="G37" s="2" t="s">
         <v>290</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D38" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="E38" s="2" t="s">
         <v>528</v>
       </c>
-      <c r="E38" s="2" t="s">
+      <c r="F38" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="F38" s="2" t="s">
+      <c r="G38" s="2" t="s">
         <v>530</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>531</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D39" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="E39" s="2" t="s">
         <v>519</v>
       </c>
-      <c r="E39" s="2" t="s">
+      <c r="F39" s="2" t="s">
         <v>520</v>
       </c>
-      <c r="F39" s="2" t="s">
+      <c r="G39" s="2" t="s">
         <v>521</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.45">
@@ -2898,7 +2906,7 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>186</v>
@@ -2907,13 +2915,13 @@
         <v>269</v>
       </c>
       <c r="E44" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="F44" s="2" t="s">
+      <c r="G44" s="2" t="s">
         <v>342</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.45">
@@ -2935,39 +2943,39 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A46" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D46" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="E46" s="2" t="s">
         <v>464</v>
       </c>
-      <c r="E46" s="2" t="s">
+      <c r="F46" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="F46" s="2" t="s">
+      <c r="G46" s="2" t="s">
         <v>466</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>467</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A47" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E47" s="2" t="s">
         <v>454</v>
       </c>
-      <c r="B47" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E47" s="2" t="s">
+      <c r="F47" s="2" t="s">
         <v>455</v>
       </c>
-      <c r="F47" s="2" t="s">
+      <c r="G47" s="2" t="s">
         <v>456</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.45">
@@ -2989,7 +2997,7 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="2" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>186</v>
@@ -2998,33 +3006,33 @@
         <v>187</v>
       </c>
       <c r="E49" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="F49" s="2" t="s">
         <v>486</v>
       </c>
-      <c r="F49" s="2" t="s">
+      <c r="G49" s="2" t="s">
         <v>487</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>488</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D50" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="E50" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="E50" s="2" t="s">
+      <c r="F50" s="2" t="s">
         <v>451</v>
       </c>
-      <c r="F50" s="2" t="s">
+      <c r="G50" s="2" t="s">
         <v>452</v>
-      </c>
-      <c r="G50" s="2" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.45">
@@ -3066,7 +3074,7 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A53" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>186</v>
@@ -3075,18 +3083,18 @@
         <v>278</v>
       </c>
       <c r="E53" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="F53" s="2" t="s">
         <v>411</v>
       </c>
-      <c r="F53" s="2" t="s">
+      <c r="G53" s="2" t="s">
         <v>412</v>
-      </c>
-      <c r="G53" s="2" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A54" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>186</v>
@@ -3095,18 +3103,18 @@
         <v>269</v>
       </c>
       <c r="E54" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="F54" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="F54" s="2" t="s">
+      <c r="G54" s="2" t="s">
         <v>307</v>
-      </c>
-      <c r="G54" s="2" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A55" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>186</v>
@@ -3115,13 +3123,13 @@
         <v>278</v>
       </c>
       <c r="E55" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="F55" s="2" t="s">
         <v>359</v>
       </c>
-      <c r="F55" s="2" t="s">
+      <c r="G55" s="2" t="s">
         <v>360</v>
-      </c>
-      <c r="G55" s="2" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.45">
@@ -3163,7 +3171,7 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>186</v>
@@ -3172,13 +3180,13 @@
         <v>269</v>
       </c>
       <c r="E58" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="F58" s="2" t="s">
         <v>474</v>
       </c>
-      <c r="F58" s="2" t="s">
+      <c r="G58" s="2" t="s">
         <v>475</v>
-      </c>
-      <c r="G58" s="2" t="s">
-        <v>476</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.45">
@@ -3200,19 +3208,19 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E60" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="B60" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E60" s="2" t="s">
+      <c r="F60" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="F60" s="2" t="s">
+      <c r="G60" s="2" t="s">
         <v>316</v>
-      </c>
-      <c r="G60" s="2" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.45">
@@ -3251,7 +3259,7 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>186</v>
@@ -3260,53 +3268,53 @@
         <v>269</v>
       </c>
       <c r="E63" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="F63" s="2" t="s">
         <v>478</v>
       </c>
-      <c r="F63" s="2" t="s">
+      <c r="G63" s="2" t="s">
         <v>479</v>
-      </c>
-      <c r="G63" s="2" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" s="2" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D64" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="E64" s="2" t="s">
         <v>440</v>
       </c>
-      <c r="E64" s="2" t="s">
+      <c r="F64" s="2" t="s">
         <v>441</v>
       </c>
-      <c r="F64" s="2" t="s">
+      <c r="G64" s="2" t="s">
         <v>442</v>
-      </c>
-      <c r="G64" s="2" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A65" s="2" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D65" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="E65" s="2" t="s">
         <v>445</v>
       </c>
-      <c r="E65" s="2" t="s">
+      <c r="F65" s="2" t="s">
         <v>446</v>
       </c>
-      <c r="F65" s="2" t="s">
+      <c r="G65" s="2" t="s">
         <v>447</v>
-      </c>
-      <c r="G65" s="2" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.45">
@@ -3328,22 +3336,22 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A67" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D67" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="E67" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="E67" s="2" t="s">
+      <c r="F67" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="F67" s="2" t="s">
+      <c r="G67" s="2" t="s">
         <v>303</v>
-      </c>
-      <c r="G67" s="2" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.45">
@@ -3419,7 +3427,7 @@
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A72" s="2" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>186</v>
@@ -3428,13 +3436,13 @@
         <v>187</v>
       </c>
       <c r="E72" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="F72" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="F72" s="2" t="s">
+      <c r="G72" s="2" t="s">
         <v>437</v>
-      </c>
-      <c r="G72" s="2" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.45">
@@ -3473,7 +3481,7 @@
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A75" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>186</v>
@@ -3482,13 +3490,13 @@
         <v>187</v>
       </c>
       <c r="E75" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="F75" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="F75" s="2" t="s">
+      <c r="G75" s="2" t="s">
         <v>403</v>
-      </c>
-      <c r="G75" s="2" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.45">
@@ -3510,19 +3518,19 @@
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A77" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>87</v>
       </c>
       <c r="E77" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="F77" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="F77" s="2" t="s">
+      <c r="G77" s="2" t="s">
         <v>421</v>
-      </c>
-      <c r="G77" s="2" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.45">
@@ -3544,101 +3552,101 @@
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A79" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D79" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="E79" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="E79" s="2" t="s">
+      <c r="F79" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="F79" s="2" t="s">
+      <c r="G79" s="2" t="s">
         <v>321</v>
-      </c>
-      <c r="G79" s="2" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A80" s="2" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D80" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="E80" s="2" t="s">
         <v>559</v>
       </c>
-      <c r="E80" s="2" t="s">
+      <c r="F80" s="2" t="s">
         <v>560</v>
       </c>
-      <c r="F80" s="2" t="s">
+      <c r="G80" s="2" t="s">
         <v>561</v>
-      </c>
-      <c r="G80" s="2" t="s">
-        <v>562</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A81" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E81" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="B81" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E81" s="2" t="s">
+      <c r="F81" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="F81" s="2" t="s">
+      <c r="G81" s="2" t="s">
         <v>399</v>
-      </c>
-      <c r="G81" s="2" t="s">
-        <v>400</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A82" s="2" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D82" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="E82" s="2" t="s">
         <v>459</v>
       </c>
-      <c r="E82" s="2" t="s">
+      <c r="F82" s="2" t="s">
         <v>460</v>
       </c>
-      <c r="F82" s="2" t="s">
+      <c r="G82" s="2" t="s">
         <v>461</v>
-      </c>
-      <c r="G82" s="2" t="s">
-        <v>462</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A83" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E83" s="2" t="s">
         <v>549</v>
       </c>
-      <c r="B83" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E83" s="2" t="s">
+      <c r="F83" s="2" t="s">
         <v>550</v>
       </c>
-      <c r="F83" s="2" t="s">
+      <c r="G83" s="2" t="s">
         <v>551</v>
-      </c>
-      <c r="G83" s="2" t="s">
-        <v>552</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A84" s="2" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>186</v>
@@ -3647,13 +3655,13 @@
         <v>269</v>
       </c>
       <c r="E84" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="F84" s="2" t="s">
         <v>498</v>
       </c>
-      <c r="F84" s="2" t="s">
+      <c r="G84" s="2" t="s">
         <v>499</v>
-      </c>
-      <c r="G84" s="2" t="s">
-        <v>500</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.45">
@@ -3675,22 +3683,22 @@
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A86" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D86" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="F86" s="2" t="s">
         <v>394</v>
       </c>
-      <c r="E86" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="F86" s="2" t="s">
+      <c r="G86" s="2" t="s">
         <v>395</v>
-      </c>
-      <c r="G86" s="2" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.45">
@@ -3729,794 +3737,780 @@
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A89" s="2" t="s">
-        <v>115</v>
+        <v>51</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>116</v>
+        <v>48</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>287</v>
+        <v>52</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>118</v>
+        <v>53</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A90" s="2" t="s">
-        <v>51</v>
+        <v>223</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>48</v>
+        <v>224</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>52</v>
+        <v>225</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>53</v>
+        <v>226</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A91" s="2" t="s">
-        <v>223</v>
+        <v>343</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>8</v>
+        <v>186</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>187</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>224</v>
+        <v>344</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>225</v>
+        <v>345</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>226</v>
+        <v>346</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A92" s="2" t="s">
-        <v>344</v>
+        <v>531</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="C92" s="2" t="s">
-        <v>187</v>
+        <v>87</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>345</v>
+        <v>532</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>346</v>
+        <v>533</v>
       </c>
       <c r="G92" s="2" t="s">
-        <v>347</v>
+        <v>534</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A93" s="2" t="s">
-        <v>532</v>
+        <v>77</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>87</v>
+        <v>8</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>533</v>
+        <v>78</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>534</v>
+        <v>79</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>535</v>
+        <v>80</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A94" s="2" t="s">
-        <v>77</v>
+        <v>227</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>78</v>
+        <v>228</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>79</v>
+        <v>229</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>80</v>
+        <v>230</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A95" s="2" t="s">
-        <v>227</v>
+        <v>39</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>228</v>
+        <v>40</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>229</v>
+        <v>41</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>230</v>
+        <v>42</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A96" s="2" t="s">
-        <v>39</v>
+        <v>295</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>40</v>
+        <v>296</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>41</v>
+        <v>297</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>42</v>
+        <v>298</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A97" s="2" t="s">
-        <v>296</v>
+        <v>143</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>297</v>
+        <v>144</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>298</v>
+        <v>145</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>299</v>
+        <v>146</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A98" s="2" t="s">
-        <v>143</v>
+        <v>81</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>8</v>
+        <v>59</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>82</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>144</v>
+        <v>83</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>145</v>
+        <v>84</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>146</v>
+        <v>85</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A99" s="2" t="s">
-        <v>81</v>
+        <v>422</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D99" s="2" t="s">
-        <v>82</v>
+        <v>186</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>187</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>83</v>
+        <v>423</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>84</v>
+        <v>424</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>85</v>
+        <v>425</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A100" s="2" t="s">
-        <v>423</v>
+        <v>54</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="C100" s="2" t="s">
-        <v>187</v>
+        <v>8</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>424</v>
+        <v>55</v>
       </c>
       <c r="F100" s="2" t="s">
-        <v>425</v>
+        <v>56</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>426</v>
+        <v>57</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A101" s="2" t="s">
-        <v>54</v>
+        <v>219</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>55</v>
+        <v>220</v>
       </c>
       <c r="F101" s="2" t="s">
-        <v>56</v>
+        <v>221</v>
       </c>
       <c r="G101" s="2" t="s">
-        <v>57</v>
+        <v>222</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A102" s="2" t="s">
-        <v>219</v>
+        <v>236</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>8</v>
+        <v>59</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>237</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>220</v>
+        <v>238</v>
       </c>
       <c r="F102" s="2" t="s">
-        <v>221</v>
+        <v>239</v>
       </c>
       <c r="G102" s="2" t="s">
-        <v>222</v>
+        <v>240</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A103" s="2" t="s">
-        <v>236</v>
+        <v>139</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D103" s="2" t="s">
-        <v>237</v>
+        <v>8</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>238</v>
+        <v>140</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>239</v>
+        <v>141</v>
       </c>
       <c r="G103" s="2" t="s">
-        <v>240</v>
+        <v>142</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A104" s="2" t="s">
-        <v>139</v>
+        <v>272</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>8</v>
+        <v>59</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>273</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>140</v>
+        <v>274</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>141</v>
+        <v>275</v>
       </c>
       <c r="G104" s="2" t="s">
-        <v>142</v>
+        <v>276</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A105" s="2" t="s">
-        <v>272</v>
+        <v>151</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D105" s="2" t="s">
-        <v>273</v>
+        <v>8</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>274</v>
+        <v>152</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>275</v>
+        <v>153</v>
       </c>
       <c r="G105" s="2" t="s">
-        <v>276</v>
+        <v>154</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A106" s="2" t="s">
-        <v>151</v>
+        <v>7</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>152</v>
+        <v>9</v>
       </c>
       <c r="F106" s="2" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="G106" s="2" t="s">
-        <v>154</v>
+        <v>11</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A107" s="2" t="s">
-        <v>7</v>
+        <v>374</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>8</v>
+        <v>59</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>375</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>9</v>
+        <v>332</v>
       </c>
       <c r="F107" s="2" t="s">
-        <v>10</v>
+        <v>376</v>
       </c>
       <c r="G107" s="2" t="s">
-        <v>11</v>
+        <v>377</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A108" s="2" t="s">
-        <v>375</v>
+        <v>500</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>376</v>
+        <v>501</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>333</v>
+        <v>502</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>377</v>
+        <v>503</v>
       </c>
       <c r="G108" s="2" t="s">
-        <v>378</v>
+        <v>504</v>
       </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A109" s="2" t="s">
-        <v>501</v>
+        <v>215</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D109" s="2" t="s">
-        <v>502</v>
+        <v>8</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>503</v>
+        <v>216</v>
       </c>
       <c r="F109" s="2" t="s">
-        <v>504</v>
+        <v>217</v>
       </c>
       <c r="G109" s="2" t="s">
-        <v>505</v>
+        <v>218</v>
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A110" s="2" t="s">
-        <v>215</v>
+        <v>31</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>216</v>
+        <v>32</v>
       </c>
       <c r="F110" s="2" t="s">
-        <v>217</v>
+        <v>33</v>
       </c>
       <c r="G110" s="2" t="s">
-        <v>218</v>
+        <v>34</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A111" s="2" t="s">
-        <v>31</v>
+        <v>176</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>32</v>
+        <v>177</v>
       </c>
       <c r="F111" s="2" t="s">
-        <v>33</v>
+        <v>178</v>
       </c>
       <c r="G111" s="2" t="s">
-        <v>34</v>
+        <v>179</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A112" s="2" t="s">
-        <v>176</v>
+        <v>522</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>177</v>
+        <v>523</v>
       </c>
       <c r="F112" s="2" t="s">
-        <v>178</v>
+        <v>524</v>
       </c>
       <c r="G112" s="2" t="s">
-        <v>179</v>
+        <v>525</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A113" s="2" t="s">
-        <v>523</v>
+        <v>365</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>8</v>
+        <v>186</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>187</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>524</v>
+        <v>366</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>525</v>
+        <v>367</v>
       </c>
       <c r="G113" s="2" t="s">
-        <v>526</v>
+        <v>368</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A114" s="2" t="s">
-        <v>366</v>
+        <v>327</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="C114" s="2" t="s">
-        <v>187</v>
+        <v>8</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>367</v>
+        <v>108</v>
       </c>
       <c r="F114" s="2" t="s">
-        <v>368</v>
+        <v>328</v>
       </c>
       <c r="G114" s="2" t="s">
-        <v>369</v>
+        <v>329</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A115" s="2" t="s">
-        <v>328</v>
+        <v>308</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>8</v>
+        <v>59</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>309</v>
       </c>
       <c r="E115" s="2" t="s">
-        <v>108</v>
+        <v>310</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>329</v>
+        <v>311</v>
       </c>
       <c r="G115" s="2" t="s">
-        <v>330</v>
+        <v>312</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A116" s="2" t="s">
-        <v>309</v>
+        <v>185</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D116" s="2" t="s">
-        <v>310</v>
+        <v>186</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>187</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>311</v>
+        <v>188</v>
       </c>
       <c r="F116" s="2" t="s">
-        <v>312</v>
+        <v>189</v>
       </c>
       <c r="G116" s="2" t="s">
-        <v>313</v>
+        <v>190</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A117" s="2" t="s">
-        <v>185</v>
+        <v>291</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>186</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>187</v>
+        <v>269</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>188</v>
+        <v>292</v>
       </c>
       <c r="F117" s="2" t="s">
-        <v>189</v>
+        <v>293</v>
       </c>
       <c r="G117" s="2" t="s">
-        <v>190</v>
+        <v>294</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A118" s="2" t="s">
-        <v>292</v>
+        <v>111</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="C118" s="2" t="s">
-        <v>269</v>
+        <v>8</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>293</v>
+        <v>112</v>
       </c>
       <c r="F118" s="2" t="s">
-        <v>294</v>
+        <v>113</v>
       </c>
       <c r="G118" s="2" t="s">
-        <v>295</v>
+        <v>114</v>
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A119" s="2" t="s">
-        <v>111</v>
+        <v>231</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>8</v>
+        <v>59</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>232</v>
       </c>
       <c r="E119" s="2" t="s">
-        <v>112</v>
+        <v>233</v>
       </c>
       <c r="F119" s="2" t="s">
-        <v>113</v>
+        <v>234</v>
       </c>
       <c r="G119" s="2" t="s">
-        <v>114</v>
+        <v>235</v>
       </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A120" s="2" t="s">
-        <v>231</v>
+        <v>480</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D120" s="2" t="s">
-        <v>232</v>
+        <v>186</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>187</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>233</v>
+        <v>481</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>234</v>
+        <v>482</v>
       </c>
       <c r="G120" s="2" t="s">
-        <v>235</v>
+        <v>483</v>
       </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A121" s="2" t="s">
-        <v>481</v>
+        <v>16</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="C121" s="2" t="s">
-        <v>187</v>
+        <v>8</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>482</v>
+        <v>13</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>483</v>
+        <v>17</v>
       </c>
       <c r="G121" s="2" t="s">
-        <v>484</v>
+        <v>18</v>
       </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A122" s="2" t="s">
-        <v>16</v>
+        <v>488</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>8</v>
+        <v>186</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>187</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>13</v>
+        <v>489</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>17</v>
+        <v>490</v>
       </c>
       <c r="G122" s="2" t="s">
-        <v>18</v>
+        <v>491</v>
       </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A123" s="2" t="s">
-        <v>489</v>
+        <v>147</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="C123" s="2" t="s">
-        <v>187</v>
+        <v>8</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>490</v>
+        <v>148</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>491</v>
+        <v>149</v>
       </c>
       <c r="G123" s="2" t="s">
-        <v>492</v>
+        <v>150</v>
       </c>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A124" s="2" t="s">
-        <v>147</v>
+        <v>413</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>8</v>
+        <v>59</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>414</v>
       </c>
       <c r="E124" s="2" t="s">
-        <v>148</v>
+        <v>415</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>149</v>
+        <v>416</v>
       </c>
       <c r="G124" s="2" t="s">
-        <v>150</v>
+        <v>417</v>
       </c>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A125" s="2" t="s">
-        <v>414</v>
+        <v>387</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>415</v>
+        <v>388</v>
       </c>
       <c r="E125" s="2" t="s">
-        <v>416</v>
+        <v>389</v>
       </c>
       <c r="F125" s="2" t="s">
-        <v>417</v>
+        <v>390</v>
       </c>
       <c r="G125" s="2" t="s">
-        <v>418</v>
+        <v>391</v>
       </c>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A126" s="2" t="s">
-        <v>388</v>
+        <v>64</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D126" s="2" t="s">
-        <v>389</v>
+        <v>8</v>
       </c>
       <c r="E126" s="2" t="s">
-        <v>390</v>
+        <v>65</v>
       </c>
       <c r="F126" s="2" t="s">
-        <v>391</v>
+        <v>66</v>
       </c>
       <c r="G126" s="2" t="s">
-        <v>392</v>
+        <v>67</v>
       </c>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A127" s="2" t="s">
-        <v>64</v>
+        <v>251</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>8</v>
+        <v>59</v>
+      </c>
+      <c r="D127" s="2" t="s">
+        <v>252</v>
       </c>
       <c r="E127" s="2" t="s">
-        <v>65</v>
+        <v>253</v>
       </c>
       <c r="F127" s="2" t="s">
-        <v>66</v>
+        <v>254</v>
       </c>
       <c r="G127" s="2" t="s">
-        <v>67</v>
+        <v>255</v>
       </c>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A128" s="2" t="s">
-        <v>251</v>
+        <v>119</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D128" s="2" t="s">
-        <v>252</v>
+        <v>8</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>253</v>
+        <v>120</v>
       </c>
       <c r="F128" s="2" t="s">
-        <v>254</v>
+        <v>121</v>
       </c>
       <c r="G128" s="2" t="s">
-        <v>255</v>
+        <v>122</v>
       </c>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A129" s="2" t="s">
-        <v>119</v>
+        <v>91</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>120</v>
+        <v>92</v>
       </c>
       <c r="F129" s="2" t="s">
-        <v>121</v>
+        <v>93</v>
       </c>
       <c r="G129" s="2" t="s">
-        <v>122</v>
+        <v>94</v>
       </c>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A130" s="2" t="s">
-        <v>91</v>
+        <v>510</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>8</v>
+        <v>59</v>
+      </c>
+      <c r="D130" s="2" t="s">
+        <v>511</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>92</v>
+        <v>253</v>
       </c>
       <c r="F130" s="2" t="s">
-        <v>93</v>
+        <v>512</v>
       </c>
       <c r="G130" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A131" s="2" t="s">
-        <v>511</v>
-      </c>
-      <c r="B131" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D131" s="2" t="s">
-        <v>512</v>
-      </c>
-      <c r="E131" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="F131" s="2" t="s">
         <v>513</v>
       </c>
-      <c r="G131" s="2" t="s">
-        <v>514</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G131" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G131">
-    <sortCondition ref="A2:A131"/>
+  <autoFilter ref="A1:G130" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G130">
+    <sortCondition ref="A2:A130"/>
   </sortState>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>